<commit_message>
Auto: Week 27/2026 data extracted from PDFs
</commit_message>
<xml_diff>
--- a/Gulf_Dashboard_W27_2026.xlsx
+++ b/Gulf_Dashboard_W27_2026.xlsx
@@ -962,26 +962,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Impact to schedule plan and delay start pile drive work
-Summary of Safety Weekly Audit issues
-Total Issues 10
-since 03 Apr 2026 - Present 18-Jun 25-Jun 2-Jul 9-Jul
-(Every Tuesday morning)
-Series1 Series2
-Safety Audit issue Status Chart
-Open Closed
-4 Environmental Impact Assessment Committee meeting. -Environment Impact At least SM ,CR and -
-Done 27 May 2026
-Assessment Committee twice a year SSHE
-5 Provide support for activities as requested by the community -School ,Government As CR -
-and Government. Agencies ,temple appropriate. Done
-6 Coordinate to participate in community activities and related -School ,Government As CR -
-government agencies Agencies ,temple appropriate. Done
-7 Strictly comply with the law. This is to prevent delays in the -Environment Impact All the Time SSHE -
-project due to complaints. Assessment Committee , Done
-Government Agencies
-Concern area of EPC
-BOP Tasks that have started and those that have not yet started are behind schedule</t>
+          <t>BOP Tasks that have started and those that have not yet started are behind schedule</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1027,26 +1008,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Delay finish of bunker foundations up to ground level. Target on PMS 07 May 2026.
-Delay finish of STG foundations up to ground level. Target on PMS 25 May 2026.
-50 Safety Weekly Audit issue
-Total Issues
-(Since 2 Apr 2026 onwards)
-Summary Safety Weekly Audit issue 6 7 Before After
-2 3 3 3 4 3 The wire of cutting equipment are Wrap with electrical tape
-Detail of reinforcement concrete duct bank of civil work.
-Detail of underground pipe of toilet at steam turbine building.
-- Owner/OE requested catch up plan of steam turbine and tipping hall.
-- Owner/OE requested to EPC to manage sequence civil work and mechanical work in boiler area.
-- Request to EPC to catch up plan. Increase man power.
-CEEC already submit catch up plan of bunker, surrounding and FGT and will submit catch up plan of tipping hall and STG
-Opened 4 issues
-No. Date of issue Discipline Subject Status
-IWTE-GSE-NCR-C-001 07/03/2026 Civil Non-conformance of Anchor bolts and Embedded parts for boiler and FGT foundation Closed
-IWTE-GSE-NCR-C-002 04/04/2026 Civil Honey combing and voids were identified after formwork removal . Open
-IWTE-GSE-NCR-C-003 24/04/2026 Civil The formwork for five(5) steam turbine foundation was removed prematurely. Open
-IWTE-GSE-NCR-C-004 19/05/2026 Civil Concrete pouring at the kicker wall of Turbine DeckMF1 Foundation Open
-IWTE-GSE-NCR-C-005 18/05/2026 Civil Improper Concrete Pouring at the wall and column Open</t>
+          <t>Detail and spec of equipment at riser pole for PEA approval.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1157,29 +1119,33 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>No cable list/schedule
-PO for cable has not been issued
-Plan Plan Actual
-No. Description Duration Actual Start Progress
-Start Finish Finish
-1 Cable duct or raceway or cable trench 1-Sep-26 30-Oct-26 60 - - -
-2 Pulling cable 1-Oct-26 10-Nov-26 40 - - -
-Concern : No manhole detail of duct bank
-Procurement process not start yet
-1 Material onsite TBC TBC - - -
-2 Installation 1-Oct 30-Nov - - -
-3 Test function TBC TBC - - -
-Concern : Procurement process not start yet
-No connection drawing
-1 Material onsite 30-Sep-26 18-Oct-26 18 - - -
-2 Installation and cable wiring 21-Sep-26 15-Oct-26 25 - - -
-3 Test function 15-Nov 6-Dec 20 - - -
-Concern : PO not submit yet
-1 Material onsite 9-Sep-26 27-Sep-26 18 - - -
-2 Installation and cable wiring 21-Sep-26 4-Oct-26 14 - - -</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
+          <t>The ZHONGHANG subcontractor selection is delayed.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>(03 Jul 26) (10 Jul 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 60.16 47.23 -12.93 67.53 49.80 -17.73 73.31
+Procurement 40% 69.36 66.35 -3.01 70.89 67.23 -3.66 72.46
+Construction 40% 9.01 10.24 1.23 10.17 11.00 0.73 11.44
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 37.36 35.36 -2.01 39.18 36.27 -2.91 40.89
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1199,26 +1165,8 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Tasks that have started and those that have not yet started are behind schedule (PMS plan).
-Impact to schedule plan and delay start pile drive work
-Safety Weekly Audit issue status by weekly
-Total Issues
-since 02 Apr 2026 - Present 10
-(Every Tuesday morning)
-18-Jun-26 25-Jun-26 2-Jul 9-Jul
-Safety Audit issue Status Chart Open Closed
-Open Closed
-and anxieties.
-Environmental Impact Assessment -Environment Impact Assessment At least twice SM ,CR and -
-Done 27 May 2026
-Committee meeting. Committee a year SSHE
-Provide support for activities as requested -School ,Government Agencies ,temple As CR -
-by the community and Government. appropriate.
-Coordinate to participate in community -School ,Government Agencies ,temple As CR -
-activities and related government agencies appropriate.
-Strictly comply with the law. This is to -Environment Impact Assessment All the Time SSHE -
-prevent delays in the project due to Committee , Government Agencies Done
-complaints.</t>
+          <t>Manpower shortage.
+BOP Tasks that have started and those that have not yet started are behind schedule</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1264,26 +1212,8 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Tasks that have started and those that have not yet started are behind schedule (PMS plan)
-Impact to schedule plan and delay start pile drive work
-Delay of work due to membrane vender shortage of workers and rain
-Safety Weekly Audit issue status by weekly
-Total Issues
-since 02 Apr 2026 - Present 20
-(Every Tuesday morning)
-18-Jun-26 25-Jun-26 2-Jul 9-Jul
-Safety Audit issue Status Chart Open Closed
-Open Closed
-and anxieties.
-Environmental Impact Assessment -Environment Impact Assessment At least twice SM ,CR and -
-Done 27 May 2026
-Committee meeting. Committee a year SSHE
-Provide support for activities as requested -School ,Government Agencies ,temple As CR -
-by the community and Government. appropriate.
-Coordinate to participate in community -School ,Government Agencies ,temple As CR -
-activities and related government agencies appropriate.
-Strictly comply with the law. This is to -Environment Impact Assessment All the Time SSHE -
-prevent delays in the project due to Committee , Government Agencies Done</t>
+          <t>Manpower shortage.
+BOP Tasks that have started and those that have not yet started are behind schedule</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1589,29 +1519,33 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>No cable list/schedule
-PO for cable has not been issued
-Plan Plan Actual
-No. Description Duration Actual Start Progress
-Start Finish Finish
-1 Cable duct or raceway or cable trench 1-Sep-26 30-Oct-26 60 - - -
-2 Pulling cable 1-Oct-26 10-Nov-26 40 - - -
-Concern : No manhole detail of duct bank
-Procurement process not start yet
-1 Material onsite TBC TBC - - -
-2 Installation 1-Oct 30-Nov - - -
-3 Test function TBC TBC - - -
-Concern : Procurement process not start yet
-No connection drawing
-1 Material onsite 30-Sep-26 18-Oct-26 18 - - -
-2 Installation and cable wiring 21-Sep-26 15-Oct-26 25 - - -
-3 Test function 15-Nov 6-Dec 20 - - -
-Concern : PO not submit yet
-1 Material onsite 9-Sep-26 27-Sep-26 18 - - -
-2 Installation and cable wiring 21-Sep-26 4-Oct-26 14 - - -</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+          <t>The ZHONGHANG subcontractor selection is delayed.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>(03 Jul 26) (10 Jul 26)
+Activities CC/SC (*)
+Plan Actual Diff. Plan Actual Diff. Acc.Plan
+% % % % % % %
+Engineering 10% 80.30 46.41 -33.89 84.08 49.81 -34.27 88.35
+Procurement 40% 74.39 72.60 -1.79 76.00 73.11 -2.89 77.49
+Construction 40% 15.69 12.74 -2.95 17.25 14.24 -3.01 18.78
+Commissioning 10% 0 0 0 0 0 0 0
+Overall 100% 44.06 38.78 -5.29 45.71 39.92 -5.79 47.34
+Safety &amp; Health :
+• Conduct SafetyToolbox Talk before starting work.
+• Mass Safety Talk at Site Area
+• Management Walk Down every Friday (10.00 – 11.00)
+• HSE Weekly Audit every Wednesday (10.00-11.00)
+• HSE Weekly Meeting with Subcontractor every Wednesday (10.00-11.00)
+• Safety Induction Training for new comers
+• Working at height Training
+Environment &amp; CoP :
+• Water spray at construction site
+• Temporary Wheel wash station</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1631,26 +1565,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Delay finish of bunker foundations up to ground level. Target on PMS 08 May 2026.
-Delay finish of STG foundations up to ground level. Target on PMS 08 Jun 2026.
-64 Safety Weekly Audit issue
-Total Issues
-(Since 2 Apr 2026 onwards) 8
-Summary Safety Weekly Audit issue 4 8 Before After
-Worker were using a damaged power The damaged power strip was
-2 4 4 strip, a potential safety hazard replaced with a new one for safe use
-Detail of reinforcement concrete duct bank of civil work.
-Detail of underground pipe of toilet at steam turbine building.
-- Owner/OE requested catch up plan of steam turbine and tipping hall.
-- Owner/OE requested to EPC to manage sequence civil work and mechanical work in boiler area.
-- Request to EPC to catch up plan and increase man power.
-CEEC already submit catch up plan of bunker, surrounding and FGT and will submit catch up plan of tipping hall and STG
-Opened 5 issues
-No. Date of issue Discipline Subject Status
-IWTE-TSE-NCR-C-001 07/03/2026 Civil Non-conformance of Anchor bolts and Embedded parts for boiler and FGT foundation Closed
-IWTE–TSE–NCR–C–002 16/03/2026 Civil Improper Concrete Pouring at the Wall of Waste Bunker Basement Open
-IWTE–TSE–NCR–C–003 21/04/2026 Civil Honey combing and voids were identified after formwork removal waste bunker column TSE . Open
-IWTE-GSE-NCR-C-004 05/05/2026 Civil Honey comb voids and concrete segregation on concrete pedestals Closed</t>
+          <t>Detail and spec of equipment at riser pole for PEA approval.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">

</xml_diff>